<commit_message>
PG - Student details updated
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git Projects\jitendrakv.github.io\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A79590-7FD3-4232-A27D-F083E1057E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D888DE50-0256-4CEB-902A-6B5E41BF593B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PhD" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="224">
   <si>
     <t>Name</t>
   </si>
@@ -671,6 +671,33 @@
   </si>
   <si>
     <t>Intelligent Approaches for Cloud Resource Provisioning</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Infosys</t>
+  </si>
+  <si>
+    <t>HSC Global</t>
+  </si>
+  <si>
+    <t>Adobe</t>
+  </si>
+  <si>
+    <t>DigiStay</t>
+  </si>
+  <si>
+    <t>MPSEDC</t>
+  </si>
+  <si>
+    <t>PhD, MANIT Bhopal</t>
+  </si>
+  <si>
+    <t>Pursuit Software</t>
+  </si>
+  <si>
+    <t>Signzy</t>
   </si>
 </sst>
 </file>
@@ -734,7 +761,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -747,7 +774,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1142,7 +1168,7 @@
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4">
         <v>2025</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -1159,7 +1185,7 @@
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5">
         <v>2025</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1196,7 +1222,7 @@
       <c r="A7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7">
         <v>2024</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1245,15 +1271,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD4758E0-2E06-CD49-AFCA-FFAEED49AC86}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K63"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="5"/>
-    <col min="5" max="5" width="111.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="0" style="5" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="0" hidden="1" customWidth="1"/>
@@ -1297,7 +1322,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -1320,7 +1345,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -1340,7 +1365,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -1360,7 +1385,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -1380,7 +1405,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1400,7 +1425,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -1420,7 +1445,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -1446,7 +1471,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>42</v>
       </c>
@@ -1472,7 +1497,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>45</v>
       </c>
@@ -1495,7 +1520,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -1514,11 +1539,14 @@
       <c r="F11" t="s">
         <v>41</v>
       </c>
+      <c r="G11" t="s">
+        <v>215</v>
+      </c>
       <c r="K11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>50</v>
       </c>
@@ -1541,7 +1569,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>52</v>
       </c>
@@ -1560,11 +1588,14 @@
       <c r="F13" t="s">
         <v>41</v>
       </c>
+      <c r="G13" t="s">
+        <v>216</v>
+      </c>
       <c r="K13" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -1583,11 +1614,14 @@
       <c r="F14" t="s">
         <v>41</v>
       </c>
+      <c r="G14" t="s">
+        <v>217</v>
+      </c>
       <c r="K14" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>55</v>
       </c>
@@ -1606,11 +1640,14 @@
       <c r="F15" t="s">
         <v>41</v>
       </c>
+      <c r="G15" t="s">
+        <v>218</v>
+      </c>
       <c r="K15" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>56</v>
       </c>
@@ -1629,11 +1666,14 @@
       <c r="F16" t="s">
         <v>41</v>
       </c>
+      <c r="G16" t="s">
+        <v>187</v>
+      </c>
       <c r="K16" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>58</v>
       </c>
@@ -1652,11 +1692,14 @@
       <c r="F17" t="s">
         <v>41</v>
       </c>
+      <c r="G17" t="s">
+        <v>221</v>
+      </c>
       <c r="K17" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -1675,11 +1718,14 @@
       <c r="F18" t="s">
         <v>41</v>
       </c>
+      <c r="G18" t="s">
+        <v>219</v>
+      </c>
       <c r="K18" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -1698,11 +1744,14 @@
       <c r="F19" t="s">
         <v>41</v>
       </c>
+      <c r="G19" t="s">
+        <v>194</v>
+      </c>
       <c r="K19" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>64</v>
       </c>
@@ -1728,7 +1777,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>66</v>
       </c>
@@ -1747,11 +1796,14 @@
       <c r="F21" t="s">
         <v>41</v>
       </c>
+      <c r="G21" t="s">
+        <v>220</v>
+      </c>
       <c r="K21" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -1777,7 +1829,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -1796,11 +1848,14 @@
       <c r="F23" t="s">
         <v>41</v>
       </c>
+      <c r="G23" t="s">
+        <v>187</v>
+      </c>
       <c r="K23" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -1819,11 +1874,14 @@
       <c r="F24" t="s">
         <v>41</v>
       </c>
+      <c r="G24" t="s">
+        <v>194</v>
+      </c>
       <c r="K24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -1842,8 +1900,11 @@
       <c r="F25" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G25" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>73</v>
       </c>
@@ -1866,7 +1927,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -1885,11 +1946,14 @@
       <c r="F27" t="s">
         <v>41</v>
       </c>
+      <c r="G27" t="s">
+        <v>222</v>
+      </c>
       <c r="K27" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>78</v>
       </c>
@@ -1908,11 +1972,14 @@
       <c r="F28" t="s">
         <v>41</v>
       </c>
+      <c r="G28" t="s">
+        <v>218</v>
+      </c>
       <c r="K28" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>80</v>
       </c>
@@ -1930,6 +1997,9 @@
       </c>
       <c r="F29" t="s">
         <v>41</v>
+      </c>
+      <c r="G29" t="s">
+        <v>223</v>
       </c>
       <c r="K29" t="s">
         <v>47</v>
@@ -1990,7 +2060,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>88</v>
       </c>
@@ -2013,7 +2083,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>90</v>
       </c>
@@ -2036,7 +2106,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>92</v>
       </c>
@@ -2059,7 +2129,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>94</v>
       </c>
@@ -2082,7 +2152,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>96</v>
       </c>
@@ -2111,7 +2181,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>98</v>
       </c>
@@ -2134,7 +2204,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>100</v>
       </c>
@@ -2157,7 +2227,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>102</v>
       </c>
@@ -2180,7 +2250,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>104</v>
       </c>
@@ -2203,7 +2273,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>106</v>
       </c>
@@ -2226,7 +2296,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>110</v>
       </c>
@@ -2292,7 +2362,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>116</v>
       </c>
@@ -2312,7 +2382,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>118</v>
       </c>
@@ -2332,7 +2402,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>120</v>
       </c>
@@ -2352,7 +2422,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>122</v>
       </c>
@@ -2372,7 +2442,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>124</v>
       </c>
@@ -2392,7 +2462,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>126</v>
       </c>
@@ -2415,7 +2485,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>128</v>
       </c>
@@ -2435,7 +2505,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>130</v>
       </c>
@@ -2455,7 +2525,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>132</v>
       </c>
@@ -2478,7 +2548,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>134</v>
       </c>
@@ -2544,7 +2614,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>139</v>
       </c>
@@ -2567,7 +2637,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>141</v>
       </c>
@@ -2587,7 +2657,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>144</v>
       </c>
@@ -2610,7 +2680,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>146</v>
       </c>
@@ -2633,7 +2703,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>148</v>
       </c>
@@ -2656,7 +2726,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>150</v>
       </c>
@@ -2703,13 +2773,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K63" xr:uid="{DD4758E0-2E06-CD49-AFCA-FFAEED49AC86}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="MSc"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K63" xr:uid="{DD4758E0-2E06-CD49-AFCA-FFAEED49AC86}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>